<commit_message>
Add anode column between category and partNumber
get_anodes() looks up the Anode component number from the same
KEMET_GOP_ATO_ANALYSIS_DAILY sheet already used for category,
keyed by PARENT_ITEM.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PW2vFyortipJRDb3aCGvTW
</commit_message>
<xml_diff>
--- a/shortage_report.xlsx
+++ b/shortage_report.xlsx
@@ -418,15 +418,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -437,25 +438,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>anode</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>partNumber</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>202634</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>matchedQty</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>gap</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Actual TPT</t>
         </is>
@@ -469,19 +475,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>A598V347M2R5AS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>T598D687M2R5ATE006</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="D2" s="1" t="n">
         <v>1060299.169066</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="E2" s="1" t="n">
         <v>926843</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="F2" s="1" t="n">
         <v>-133456.169066</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>21.47815950920245</v>
       </c>
     </row>
@@ -493,19 +504,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>A520V337M003ASMHSP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>T520V337M2R5ATE025</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="D3" s="1" t="n">
         <v>15447.605017</v>
       </c>
-      <c r="D3" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
         <v>-15447.605017</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>17.506</v>
       </c>
     </row>
@@ -517,19 +533,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>A520D337M006ASMHSP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>T520D337M006ATE018</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>16.84041666666666</v>
       </c>
     </row>
@@ -541,19 +562,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>A520V157M006ASE007</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>T520D157M006ATE009E007</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="D5" s="1" t="n">
         <v>1637.736953</v>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="n">
         <v>-1637.736953</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>19.90666666666667</v>
       </c>
     </row>
@@ -565,19 +591,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>A520V477M003ASMHSP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>T520V477M2R5ATE018</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="D6" s="1" t="n">
         <v>181558.102884</v>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="E6" s="1" t="n">
         <v>131718</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="F6" s="1" t="n">
         <v>-49840.10288399999</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>17.50933884297521</v>
       </c>
     </row>
@@ -589,19 +620,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>A520D227M010ASMHSB</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>T520D227M010ATE018</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>14.43026041666667</v>
       </c>
     </row>
@@ -613,19 +649,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>A520B227M006ASALT1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>T520B227M006ATE035</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D8" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>13.60854166666667</v>
       </c>
     </row>
@@ -637,19 +678,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>A520B107M006ASE018</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>T520B107M006ATE018</t>
         </is>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="D9" s="1" t="n">
         <v>5015.32295</v>
       </c>
-      <c r="D9" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1" t="n">
         <v>-5015.32295</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>19.20604166666667</v>
       </c>
     </row>
@@ -661,19 +707,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>A520V107M010ASE009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>T520V107M006ATE009E007</t>
         </is>
       </c>
-      <c r="C10" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>22.4775</v>
       </c>
     </row>
@@ -685,19 +736,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>A520D337M006ASE010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>T520D337M006ATE009</t>
         </is>
       </c>
-      <c r="C11" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>18.59724550898204</v>
       </c>
     </row>
@@ -709,19 +765,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>A521D227M016AS</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>T521D227M016ATE035</t>
         </is>
       </c>
-      <c r="C12" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>16.085</v>
       </c>
     </row>
@@ -733,19 +794,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>A598V247M004AS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>T598D477M2R5ATE0067280</t>
         </is>
       </c>
-      <c r="C13" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>19.5720942408377</v>
       </c>
     </row>
@@ -757,19 +823,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>A520V477M006ASMHSP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>T520V477M006ATE055</t>
         </is>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="D14" s="1" t="n">
         <v>1361.377465</v>
       </c>
-      <c r="D14" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1" t="n">
         <v>-1361.377465</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>18.434</v>
       </c>
     </row>
@@ -781,19 +852,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>A520B227M2R5ASE021</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>T520B227M2R5ATE015</t>
         </is>
       </c>
-      <c r="C15" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>16.91601851851852</v>
       </c>
     </row>
@@ -805,19 +881,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>A520D477M004ASE012</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>T520D477M004ATE012</t>
         </is>
       </c>
-      <c r="C16" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D16" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="n">
         <v>16.01483870967742</v>
       </c>
     </row>
@@ -829,19 +910,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>A521D107M025ASALT2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>T521D107M025ATE0407280</t>
         </is>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="D17" s="1" t="n">
         <v>3948929.81405</v>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="E17" s="1" t="n">
         <v>1499228</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="F17" s="1" t="n">
         <v>-2449701.81405</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>11.93435144609988</v>
       </c>
     </row>
@@ -853,19 +939,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>A520V107M010ASMHSB</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>T520V107M010ATE018</t>
         </is>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="D18" s="1" t="n">
         <v>115756.818077</v>
       </c>
-      <c r="D18" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1" t="n">
         <v>-115756.818077</v>
       </c>
-      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -875,19 +966,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>A521V107M020ASMH01</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>T521V107M020ATE055</t>
         </is>
       </c>
-      <c r="C19" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D19" s="1" t="n">
-        <v>797722</v>
+        <v>0</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>797722</v>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="F19" s="1" t="n">
+        <v>797722</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>15.04557425742575</v>
       </c>
     </row>
@@ -899,19 +995,24 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>A520V477M006ASMHSP</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>T520V477M006ATE035</t>
         </is>
       </c>
-      <c r="C20" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2" t="n">
         <v>19.46818181818182</v>
       </c>
     </row>
@@ -923,19 +1024,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>A528B906M002ASE006</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>T528B277M002APE006</t>
         </is>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="D21" s="1" t="n">
         <v>185610.378537</v>
       </c>
-      <c r="D21" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1" t="n">
         <v>-185610.378537</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>36.352</v>
       </c>
     </row>
@@ -947,19 +1053,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>A528Z477M003ASE009</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>T528Z477M2R5ATE009E008</t>
         </is>
       </c>
-      <c r="C22" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D22" s="1" t="n">
-        <v>67184</v>
+        <v>0</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>67184</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="1" t="n">
+        <v>67184</v>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>33.7525</v>
       </c>
     </row>
@@ -971,19 +1082,24 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>A521B106M035AS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>T521B106M035ATE200</t>
         </is>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="D23" s="1" t="n">
         <v>8786.043369999999</v>
       </c>
-      <c r="D23" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1" t="n">
         <v>-8786.043369999999</v>
       </c>
-      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -993,19 +1109,24 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>A530V157M2R5ASE005</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>T530D477M2R5ATE005</t>
         </is>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="D24" s="1" t="n">
         <v>5421.686748</v>
       </c>
-      <c r="D24" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="1" t="n">
         <v>-5421.686748</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="G24" s="2" t="n">
         <v>19.66</v>
       </c>
     </row>
@@ -1017,19 +1138,24 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>A521V107M016ASMHSP</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>T521V107M016ATE040</t>
         </is>
       </c>
-      <c r="C25" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="F25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
         <v>15.12</v>
       </c>
     </row>
@@ -1041,19 +1167,24 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>A530V157M006ASE004</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>T530X477M006ATE004</t>
         </is>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="D26" s="1" t="n">
         <v>30835.536948</v>
       </c>
-      <c r="D26" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="1" t="n">
         <v>-30835.536948</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>18.8862</v>
       </c>
     </row>
@@ -1065,19 +1196,24 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>A521V476M016ASMHSP</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>T521V476M016ATE040</t>
         </is>
       </c>
-      <c r="C27" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D27" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="F27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="n">
         <v>12.52</v>
       </c>
     </row>
@@ -1089,19 +1225,24 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>A598V247M004AS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>T598D477M2R5ATE006</t>
         </is>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="D28" s="1" t="n">
         <v>1209358.95066</v>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="E28" s="1" t="n">
         <v>591038</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="F28" s="1" t="n">
         <v>-618320.9506600001</v>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>19.67699029126213</v>
       </c>
     </row>
@@ -1113,19 +1254,24 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>A521V157M016AS</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>T521V157M016ATE050</t>
         </is>
       </c>
-      <c r="C29" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="F29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="n">
         <v>17.25547619047619</v>
       </c>
     </row>
@@ -1137,19 +1283,24 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>A521V685M063ASSUZH</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
           <t>T521X226M063ATE075</t>
         </is>
       </c>
-      <c r="C30" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D30" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="n">
         <v>20.32785714285714</v>
       </c>
     </row>
@@ -1161,19 +1312,24 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>A521V476M016ASMHSP</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
           <t>T521V476M016ATE070</t>
         </is>
       </c>
-      <c r="C31" s="1" t="n">
+      <c r="D31" s="1" t="n">
         <v>31567.049544</v>
       </c>
-      <c r="D31" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="1" t="n">
         <v>-31567.049544</v>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>14.37666666666667</v>
       </c>
     </row>
@@ -1185,19 +1341,24 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>A521V247M016ASMHSP</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
           <t>T521X477M016ATE020</t>
         </is>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="D32" s="1" t="n">
         <v>107154.090896</v>
       </c>
-      <c r="D32" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="1" t="n">
         <v>-107154.090896</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>17.16212765957447</v>
       </c>
     </row>
@@ -1209,19 +1370,24 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>A528Z337M003ASE009</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>T528Z337M2R5ATE009E008</t>
         </is>
       </c>
-      <c r="C33" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
         <v>33.815</v>
       </c>
     </row>
@@ -1233,39 +1399,45 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>A520B227M006ASALT1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
           <t>T520B227M006ATE045</t>
         </is>
       </c>
-      <c r="C34" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D34" s="1" t="n">
-        <v>102000</v>
+        <v>0</v>
       </c>
       <c r="E34" s="1" t="n">
         <v>102000</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F34" s="1" t="n">
+        <v>102000</v>
+      </c>
+      <c r="G34" s="2" t="n">
         <v>13.93418198529412</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr">
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
         <is>
           <t>T520X337M010ATE010</t>
         </is>
       </c>
-      <c r="C35" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D35" s="1" t="n">
-        <v>268557</v>
+        <v>0</v>
       </c>
       <c r="E35" s="1" t="n">
         <v>268557</v>
       </c>
-      <c r="F35" s="2" t="n"/>
+      <c r="F35" s="1" t="n">
+        <v>268557</v>
+      </c>
+      <c r="G35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1275,19 +1447,24 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>A530V117M010ASE004</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>T530X337M010ATE004</t>
         </is>
       </c>
-      <c r="C36" s="1" t="n">
+      <c r="D36" s="1" t="n">
         <v>7492.265061</v>
       </c>
-      <c r="D36" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E36" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="1" t="n">
         <v>-7492.265061</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>20.47947368421053</v>
       </c>
     </row>
@@ -1299,19 +1476,24 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>A530V227M004ASE004</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
           <t>T530X687M004ATE004</t>
         </is>
       </c>
-      <c r="C37" s="1" t="n">
+      <c r="D37" s="1" t="n">
         <v>15400.177233</v>
       </c>
-      <c r="D37" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E37" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="1" t="n">
         <v>-15400.177233</v>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>22.53768115942029</v>
       </c>
     </row>
@@ -1323,19 +1505,24 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>A598V247M004AS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
           <t>T598D477M2R5AT4186</t>
         </is>
       </c>
-      <c r="C38" s="1" t="n">
+      <c r="D38" s="1" t="n">
         <v>36969.354132</v>
       </c>
-      <c r="D38" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E38" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="1" t="n">
         <v>-36969.354132</v>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="G38" s="2" t="n">
         <v>20.37757575757576</v>
       </c>
     </row>
@@ -1347,19 +1534,24 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>A530V117M010ASE006</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
           <t>T530X337M010AHE006</t>
         </is>
       </c>
-      <c r="C39" s="1" t="n">
+      <c r="D39" s="1" t="n">
         <v>5101.127334000001</v>
       </c>
-      <c r="D39" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E39" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="1" t="n">
         <v>-5101.127334000001</v>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>18.875</v>
       </c>
     </row>
@@ -1371,19 +1563,24 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>A520V107M010ASMHSP</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
           <t>T520V107M010ATE0502478</t>
         </is>
       </c>
-      <c r="C40" s="1" t="n">
+      <c r="D40" s="1" t="n">
         <v>5669.429191</v>
       </c>
-      <c r="D40" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="1" t="n">
         <v>-5669.429191</v>
       </c>
-      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1393,19 +1590,24 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>A520V107M010ASMHSP</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
           <t>T520V107M010ATE025</t>
         </is>
       </c>
-      <c r="C41" s="1" t="n">
+      <c r="D41" s="1" t="n">
         <v>10131.826318</v>
       </c>
-      <c r="D41" s="1" t="n">
+      <c r="E41" s="1" t="n">
         <v>45066</v>
       </c>
-      <c r="E41" s="1" t="n">
+      <c r="F41" s="1" t="n">
         <v>34934.173682</v>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>18.425</v>
       </c>
     </row>
@@ -1417,19 +1619,24 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>A520B107M006ASE025</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
           <t>T520B107M006ATE025</t>
         </is>
       </c>
-      <c r="C42" s="1" t="n">
+      <c r="D42" s="1" t="n">
         <v>297872.79306</v>
       </c>
-      <c r="D42" s="1" t="n">
+      <c r="E42" s="1" t="n">
         <v>304191</v>
       </c>
-      <c r="E42" s="1" t="n">
+      <c r="F42" s="1" t="n">
         <v>6318.206940000004</v>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>12.53888888888889</v>
       </c>
     </row>
@@ -1441,19 +1648,24 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>A521D107M025ASMHSP</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
           <t>T521D107M025ATE040</t>
         </is>
       </c>
-      <c r="C43" s="1" t="n">
+      <c r="D43" s="1" t="n">
         <v>139986.564337</v>
       </c>
-      <c r="D43" s="1" t="n">
+      <c r="E43" s="1" t="n">
         <v>115534</v>
       </c>
-      <c r="E43" s="1" t="n">
+      <c r="F43" s="1" t="n">
         <v>-24452.56433700002</v>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="G43" s="2" t="n">
         <v>12.48259717314488</v>
       </c>
     </row>
@@ -1465,19 +1677,24 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>A530V117M010ASE004</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
           <t>T530X337M010ATE005</t>
         </is>
       </c>
-      <c r="C44" s="1" t="n">
+      <c r="D44" s="1" t="n">
         <v>68379</v>
       </c>
-      <c r="D44" s="1" t="n">
+      <c r="E44" s="1" t="n">
         <v>66593</v>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="F44" s="1" t="n">
         <v>-1786</v>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="G44" s="2" t="n">
         <v>19.49571428571429</v>
       </c>
     </row>
@@ -1492,15 +1709,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1511,25 +1729,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>anode</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>partNumber</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>202634</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>matchedQty</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>gap</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Actual TPT</t>
         </is>
@@ -1543,19 +1766,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>A598V347M2R5AS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>T598D687M2R5ATE006</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="D2" s="1" t="n">
         <v>1060299.169066</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="E2" s="1" t="n">
         <v>926843</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="F2" s="1" t="n">
         <v>-133456.169066</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>21.47815950920245</v>
       </c>
     </row>
@@ -1567,19 +1795,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>A520V337M003ASMHSP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>T520V337M2R5ATE025</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="D3" s="1" t="n">
         <v>15447.605017</v>
       </c>
-      <c r="D3" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
         <v>-15447.605017</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>17.506</v>
       </c>
     </row>
@@ -1591,19 +1824,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>A520V157M006ASE007</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>T520D157M006ATE009E007</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="D4" s="1" t="n">
         <v>1637.736953</v>
       </c>
-      <c r="D4" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="n">
         <v>-1637.736953</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>19.90666666666667</v>
       </c>
     </row>
@@ -1615,19 +1853,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>A520V477M003ASMHSP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>T520V477M2R5ATE018</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="D5" s="1" t="n">
         <v>181558.102884</v>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="E5" s="1" t="n">
         <v>131718</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="F5" s="1" t="n">
         <v>-49840.10288399999</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>17.50933884297521</v>
       </c>
     </row>
@@ -1639,19 +1882,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>A520B107M006ASE018</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>T520B107M006ATE018</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="D6" s="1" t="n">
         <v>5015.32295</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="n">
         <v>-5015.32295</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>19.20604166666667</v>
       </c>
     </row>
@@ -1663,19 +1911,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>A520V477M006ASMHSP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>T520V477M006ATE055</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="D7" s="1" t="n">
         <v>1361.377465</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="n">
         <v>-1361.377465</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>18.434</v>
       </c>
     </row>
@@ -1687,19 +1940,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>A521D107M025ASALT2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>T521D107M025ATE0407280</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="D8" s="1" t="n">
         <v>3948929.81405</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="E8" s="1" t="n">
         <v>1499228</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="F8" s="1" t="n">
         <v>-2449701.81405</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>11.93435144609988</v>
       </c>
     </row>
@@ -1711,19 +1969,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>A520V107M010ASMHSB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>T520V107M010ATE018</t>
         </is>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="D9" s="1" t="n">
         <v>115756.818077</v>
       </c>
-      <c r="D9" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1" t="n">
         <v>-115756.818077</v>
       </c>
-      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1733,19 +1996,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>A528B906M002ASE006</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>T528B277M002APE006</t>
         </is>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="D10" s="1" t="n">
         <v>185610.378537</v>
       </c>
-      <c r="D10" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1" t="n">
         <v>-185610.378537</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>36.352</v>
       </c>
     </row>
@@ -1757,19 +2025,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>A521B106M035AS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>T521B106M035ATE200</t>
         </is>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="D11" s="1" t="n">
         <v>8786.043369999999</v>
       </c>
-      <c r="D11" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1" t="n">
         <v>-8786.043369999999</v>
       </c>
-      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1779,19 +2052,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>A530V157M2R5ASE005</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>T530D477M2R5ATE005</t>
         </is>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="D12" s="1" t="n">
         <v>5421.686748</v>
       </c>
-      <c r="D12" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1" t="n">
         <v>-5421.686748</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>19.66</v>
       </c>
     </row>
@@ -1803,19 +2081,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>A530V157M006ASE004</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>T530X477M006ATE004</t>
         </is>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="D13" s="1" t="n">
         <v>30835.536948</v>
       </c>
-      <c r="D13" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1" t="n">
         <v>-30835.536948</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>18.8862</v>
       </c>
     </row>
@@ -1827,19 +2110,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>A598V247M004AS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>T598D477M2R5ATE006</t>
         </is>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="D14" s="1" t="n">
         <v>1209358.95066</v>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="E14" s="1" t="n">
         <v>591038</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="F14" s="1" t="n">
         <v>-618320.9506600001</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>19.67699029126213</v>
       </c>
     </row>
@@ -1851,19 +2139,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>A521V476M016ASMHSP</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>T521V476M016ATE070</t>
         </is>
       </c>
-      <c r="C15" s="1" t="n">
+      <c r="D15" s="1" t="n">
         <v>31567.049544</v>
       </c>
-      <c r="D15" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="1" t="n">
         <v>-31567.049544</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>14.37666666666667</v>
       </c>
     </row>
@@ -1875,19 +2168,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>A521V247M016ASMHSP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>T521X477M016ATE020</t>
         </is>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="D16" s="1" t="n">
         <v>107154.090896</v>
       </c>
-      <c r="D16" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1" t="n">
         <v>-107154.090896</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>17.16212765957447</v>
       </c>
     </row>
@@ -1899,19 +2197,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>A530V117M010ASE004</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>T530X337M010ATE004</t>
         </is>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="D17" s="1" t="n">
         <v>7492.265061</v>
       </c>
-      <c r="D17" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1" t="n">
         <v>-7492.265061</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>20.47947368421053</v>
       </c>
     </row>
@@ -1923,19 +2226,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>A530V227M004ASE004</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>T530X687M004ATE004</t>
         </is>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="D18" s="1" t="n">
         <v>15400.177233</v>
       </c>
-      <c r="D18" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1" t="n">
         <v>-15400.177233</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>22.53768115942029</v>
       </c>
     </row>
@@ -1947,19 +2255,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>A598V247M004AS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>T598D477M2R5AT4186</t>
         </is>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="D19" s="1" t="n">
         <v>36969.354132</v>
       </c>
-      <c r="D19" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1" t="n">
         <v>-36969.354132</v>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>20.37757575757576</v>
       </c>
     </row>
@@ -1971,19 +2284,24 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>A530V117M010ASE006</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>T530X337M010AHE006</t>
         </is>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="D20" s="1" t="n">
         <v>5101.127334000001</v>
       </c>
-      <c r="D20" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="1" t="n">
         <v>-5101.127334000001</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>18.875</v>
       </c>
     </row>
@@ -1995,19 +2313,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>A520V107M010ASMHSP</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>T520V107M010ATE0502478</t>
         </is>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="D21" s="1" t="n">
         <v>5669.429191</v>
       </c>
-      <c r="D21" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1" t="n">
         <v>-5669.429191</v>
       </c>
-      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2017,19 +2340,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>A521D107M025ASMHSP</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>T521D107M025ATE040</t>
         </is>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="D22" s="1" t="n">
         <v>139986.564337</v>
       </c>
-      <c r="D22" s="1" t="n">
+      <c r="E22" s="1" t="n">
         <v>115534</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="F22" s="1" t="n">
         <v>-24452.56433700002</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>12.48259717314488</v>
       </c>
     </row>
@@ -2041,19 +2369,24 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>A530V117M010ASE004</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>T530X337M010ATE005</t>
         </is>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="D23" s="1" t="n">
         <v>68379</v>
       </c>
-      <c r="D23" s="1" t="n">
+      <c r="E23" s="1" t="n">
         <v>66593</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="F23" s="1" t="n">
         <v>-1786</v>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>19.49571428571429</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Need By Date column for the shortage
Earliest NEED_BY_DATE from KEMET_GOP_ATO_ANALYSIS_DAILY, keyed by
PARENT_ITEM, as confirmed with the user: the shortage's completion
date comes from NEED_BY_DATE (the demand's due date), taking the
earliest one since a partNumber spans many order lines with differing
dates.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PW2vFyortipJRDb3aCGvTW
</commit_message>
<xml_diff>
--- a/shortage_report.xlsx
+++ b/shortage_report.xlsx
@@ -17,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;(#,##0)"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,10 +51,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -428,6 +431,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,6 +470,11 @@
           <t>Actual TPT</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Need By Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -495,6 +504,9 @@
       <c r="G2" s="2" t="n">
         <v>21.47815950920245</v>
       </c>
+      <c r="H2" s="3" t="n">
+        <v>46293</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -524,6 +536,9 @@
       <c r="G3" s="2" t="n">
         <v>17.506</v>
       </c>
+      <c r="H3" s="3" t="n">
+        <v>46278</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -553,6 +568,9 @@
       <c r="G4" s="2" t="n">
         <v>16.84041666666666</v>
       </c>
+      <c r="H4" s="3" t="n">
+        <v>46279</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -582,6 +600,9 @@
       <c r="G5" s="2" t="n">
         <v>19.90666666666667</v>
       </c>
+      <c r="H5" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -611,6 +632,9 @@
       <c r="G6" s="2" t="n">
         <v>17.50933884297521</v>
       </c>
+      <c r="H6" s="3" t="n">
+        <v>46278</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -640,6 +664,9 @@
       <c r="G7" s="2" t="n">
         <v>14.43026041666667</v>
       </c>
+      <c r="H7" s="3" t="n">
+        <v>46278</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -669,6 +696,9 @@
       <c r="G8" s="2" t="n">
         <v>13.60854166666667</v>
       </c>
+      <c r="H8" s="3" t="n">
+        <v>46274</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -698,6 +728,9 @@
       <c r="G9" s="2" t="n">
         <v>19.20604166666667</v>
       </c>
+      <c r="H9" s="3" t="n">
+        <v>46270</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -727,6 +760,9 @@
       <c r="G10" s="2" t="n">
         <v>22.4775</v>
       </c>
+      <c r="H10" s="3" t="n">
+        <v>46284</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -756,6 +792,9 @@
       <c r="G11" s="2" t="n">
         <v>18.59724550898204</v>
       </c>
+      <c r="H11" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -785,6 +824,9 @@
       <c r="G12" s="2" t="n">
         <v>16.085</v>
       </c>
+      <c r="H12" s="3" t="n">
+        <v>46279</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -814,6 +856,9 @@
       <c r="G13" s="2" t="n">
         <v>19.5720942408377</v>
       </c>
+      <c r="H13" s="3" t="n">
+        <v>46287</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -843,6 +888,9 @@
       <c r="G14" s="2" t="n">
         <v>18.434</v>
       </c>
+      <c r="H14" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -872,6 +920,9 @@
       <c r="G15" s="2" t="n">
         <v>16.91601851851852</v>
       </c>
+      <c r="H15" s="3" t="n">
+        <v>46279</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -901,6 +952,9 @@
       <c r="G16" s="2" t="n">
         <v>16.01483870967742</v>
       </c>
+      <c r="H16" s="3" t="n">
+        <v>46279</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -930,6 +984,9 @@
       <c r="G17" s="2" t="n">
         <v>11.93435144609988</v>
       </c>
+      <c r="H17" s="3" t="n">
+        <v>46272</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -957,6 +1014,9 @@
         <v>-115756.818077</v>
       </c>
       <c r="G18" s="2" t="n"/>
+      <c r="H18" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -986,6 +1046,9 @@
       <c r="G19" s="2" t="n">
         <v>15.04557425742575</v>
       </c>
+      <c r="H19" s="3" t="n">
+        <v>46281</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1015,6 +1078,9 @@
       <c r="G20" s="2" t="n">
         <v>19.46818181818182</v>
       </c>
+      <c r="H20" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1044,6 +1110,9 @@
       <c r="G21" s="2" t="n">
         <v>36.352</v>
       </c>
+      <c r="H21" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1073,6 +1142,9 @@
       <c r="G22" s="2" t="n">
         <v>33.7525</v>
       </c>
+      <c r="H22" s="3" t="n">
+        <v>46293</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1100,6 +1172,9 @@
         <v>-8786.043369999999</v>
       </c>
       <c r="G23" s="2" t="n"/>
+      <c r="H23" s="3" t="n">
+        <v>46266</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1129,6 +1204,9 @@
       <c r="G24" s="2" t="n">
         <v>19.66</v>
       </c>
+      <c r="H24" s="3" t="n">
+        <v>46279</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1158,6 +1236,9 @@
       <c r="G25" s="2" t="n">
         <v>15.12</v>
       </c>
+      <c r="H25" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1187,6 +1268,9 @@
       <c r="G26" s="2" t="n">
         <v>18.8862</v>
       </c>
+      <c r="H26" s="3" t="n">
+        <v>46278</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1216,6 +1300,9 @@
       <c r="G27" s="2" t="n">
         <v>12.52</v>
       </c>
+      <c r="H27" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1245,6 +1332,9 @@
       <c r="G28" s="2" t="n">
         <v>19.67699029126213</v>
       </c>
+      <c r="H28" s="3" t="n">
+        <v>46281</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1274,6 +1364,9 @@
       <c r="G29" s="2" t="n">
         <v>17.25547619047619</v>
       </c>
+      <c r="H29" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1303,6 +1396,9 @@
       <c r="G30" s="2" t="n">
         <v>20.32785714285714</v>
       </c>
+      <c r="H30" s="3" t="n">
+        <v>46287</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1332,6 +1428,9 @@
       <c r="G31" s="2" t="n">
         <v>14.37666666666667</v>
       </c>
+      <c r="H31" s="3" t="n">
+        <v>46274</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1361,6 +1460,9 @@
       <c r="G32" s="2" t="n">
         <v>17.16212765957447</v>
       </c>
+      <c r="H32" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1390,6 +1492,9 @@
       <c r="G33" s="2" t="n">
         <v>33.815</v>
       </c>
+      <c r="H33" s="3" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1418,6 +1523,9 @@
       </c>
       <c r="G34" s="2" t="n">
         <v>13.93418198529412</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>46274</v>
       </c>
     </row>
     <row r="35">
@@ -1438,6 +1546,7 @@
         <v>268557</v>
       </c>
       <c r="G35" s="2" t="n"/>
+      <c r="H35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1467,6 +1576,9 @@
       <c r="G36" s="2" t="n">
         <v>20.47947368421053</v>
       </c>
+      <c r="H36" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1496,6 +1608,9 @@
       <c r="G37" s="2" t="n">
         <v>22.53768115942029</v>
       </c>
+      <c r="H37" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1525,6 +1640,9 @@
       <c r="G38" s="2" t="n">
         <v>20.37757575757576</v>
       </c>
+      <c r="H38" s="3" t="n">
+        <v>46285</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1554,6 +1672,9 @@
       <c r="G39" s="2" t="n">
         <v>18.875</v>
       </c>
+      <c r="H39" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1581,6 +1702,9 @@
         <v>-5669.429191</v>
       </c>
       <c r="G40" s="2" t="n"/>
+      <c r="H40" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1610,6 +1734,9 @@
       <c r="G41" s="2" t="n">
         <v>18.425</v>
       </c>
+      <c r="H41" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1639,6 +1766,9 @@
       <c r="G42" s="2" t="n">
         <v>12.53888888888889</v>
       </c>
+      <c r="H42" s="3" t="n">
+        <v>46273</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1668,6 +1798,9 @@
       <c r="G43" s="2" t="n">
         <v>12.48259717314488</v>
       </c>
+      <c r="H43" s="3" t="n">
+        <v>46274</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1696,6 +1829,9 @@
       </c>
       <c r="G44" s="2" t="n">
         <v>19.49571428571429</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>46277</v>
       </c>
     </row>
   </sheetData>
@@ -1709,7 +1845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1719,6 +1855,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1757,6 +1894,11 @@
           <t>Actual TPT</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Need By Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1786,6 +1928,9 @@
       <c r="G2" s="2" t="n">
         <v>21.47815950920245</v>
       </c>
+      <c r="H2" s="3" t="n">
+        <v>46293</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1815,6 +1960,9 @@
       <c r="G3" s="2" t="n">
         <v>17.506</v>
       </c>
+      <c r="H3" s="3" t="n">
+        <v>46278</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1844,6 +1992,9 @@
       <c r="G4" s="2" t="n">
         <v>19.90666666666667</v>
       </c>
+      <c r="H4" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1873,6 +2024,9 @@
       <c r="G5" s="2" t="n">
         <v>17.50933884297521</v>
       </c>
+      <c r="H5" s="3" t="n">
+        <v>46278</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1902,6 +2056,9 @@
       <c r="G6" s="2" t="n">
         <v>19.20604166666667</v>
       </c>
+      <c r="H6" s="3" t="n">
+        <v>46270</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1931,6 +2088,9 @@
       <c r="G7" s="2" t="n">
         <v>18.434</v>
       </c>
+      <c r="H7" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1960,6 +2120,9 @@
       <c r="G8" s="2" t="n">
         <v>11.93435144609988</v>
       </c>
+      <c r="H8" s="3" t="n">
+        <v>46272</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1987,6 +2150,9 @@
         <v>-115756.818077</v>
       </c>
       <c r="G9" s="2" t="n"/>
+      <c r="H9" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2016,6 +2182,9 @@
       <c r="G10" s="2" t="n">
         <v>36.352</v>
       </c>
+      <c r="H10" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2043,6 +2212,9 @@
         <v>-8786.043369999999</v>
       </c>
       <c r="G11" s="2" t="n"/>
+      <c r="H11" s="3" t="n">
+        <v>46266</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2072,6 +2244,9 @@
       <c r="G12" s="2" t="n">
         <v>19.66</v>
       </c>
+      <c r="H12" s="3" t="n">
+        <v>46279</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2101,6 +2276,9 @@
       <c r="G13" s="2" t="n">
         <v>18.8862</v>
       </c>
+      <c r="H13" s="3" t="n">
+        <v>46278</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2130,6 +2308,9 @@
       <c r="G14" s="2" t="n">
         <v>19.67699029126213</v>
       </c>
+      <c r="H14" s="3" t="n">
+        <v>46281</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2159,6 +2340,9 @@
       <c r="G15" s="2" t="n">
         <v>14.37666666666667</v>
       </c>
+      <c r="H15" s="3" t="n">
+        <v>46274</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2188,6 +2372,9 @@
       <c r="G16" s="2" t="n">
         <v>17.16212765957447</v>
       </c>
+      <c r="H16" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2217,6 +2404,9 @@
       <c r="G17" s="2" t="n">
         <v>20.47947368421053</v>
       </c>
+      <c r="H17" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2246,6 +2436,9 @@
       <c r="G18" s="2" t="n">
         <v>22.53768115942029</v>
       </c>
+      <c r="H18" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2275,6 +2468,9 @@
       <c r="G19" s="2" t="n">
         <v>20.37757575757576</v>
       </c>
+      <c r="H19" s="3" t="n">
+        <v>46285</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2304,6 +2500,9 @@
       <c r="G20" s="2" t="n">
         <v>18.875</v>
       </c>
+      <c r="H20" s="3" t="n">
+        <v>46280</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2331,6 +2530,9 @@
         <v>-5669.429191</v>
       </c>
       <c r="G21" s="2" t="n"/>
+      <c r="H21" s="3" t="n">
+        <v>46277</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2360,6 +2562,9 @@
       <c r="G22" s="2" t="n">
         <v>12.48259717314488</v>
       </c>
+      <c r="H22" s="3" t="n">
+        <v>46274</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2388,6 +2593,9 @@
       </c>
       <c r="G23" s="2" t="n">
         <v>19.49571428571429</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>46277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>